<commit_message>
feat: update payment template with new structure and formatting
</commit_message>
<xml_diff>
--- a/backend/server/templates/payment-template.xlsx
+++ b/backend/server/templates/payment-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Desktop\own_pr\Kr\web-kr\backend\server\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C68F307-15F6-4E7E-9BC8-E1FB83E513D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{262D71EA-F52D-48A7-814E-CE08AD842B83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{3923C61F-7339-427F-A90F-C317D1518F14}"/>
   </bookViews>
@@ -440,7 +440,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -466,21 +466,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -511,26 +499,44 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="left" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" shrinkToFit="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -850,50 +856,51 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.77734375" customWidth="1"/>
-    <col min="2" max="3" width="13.77734375" customWidth="1"/>
+    <col min="2" max="2" width="10.77734375" customWidth="1"/>
+    <col min="3" max="3" width="13.77734375" customWidth="1"/>
     <col min="4" max="4" width="15.88671875" customWidth="1"/>
     <col min="5" max="5" width="10.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="7.77734375" customWidth="1"/>
-    <col min="13" max="13" width="13.77734375" customWidth="1"/>
+    <col min="13" max="13" width="10.77734375" customWidth="1"/>
     <col min="16" max="16" width="10.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="26"/>
-      <c r="I1" s="26"/>
-      <c r="J1" s="26"/>
-      <c r="K1" s="26"/>
-      <c r="L1" s="26"/>
-      <c r="M1" s="26"/>
-      <c r="N1" s="26"/>
-      <c r="O1" s="26"/>
-      <c r="P1" s="27"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
+      <c r="K1" s="21"/>
+      <c r="L1" s="21"/>
+      <c r="M1" s="21"/>
+      <c r="N1" s="21"/>
+      <c r="O1" s="21"/>
+      <c r="P1" s="22"/>
       <c r="Q1" s="1"/>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A2" s="28" t="s">
+      <c r="A2" s="27" t="s">
         <v>29</v>
       </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
       <c r="E2" s="1"/>
-      <c r="F2" s="30" t="s">
+      <c r="F2" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
-      <c r="I2" s="30"/>
-      <c r="J2" s="30"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="25"/>
+      <c r="I2" s="25"/>
+      <c r="J2" s="25"/>
       <c r="K2" s="1"/>
       <c r="L2" s="1"/>
       <c r="M2" s="1"/>
@@ -903,21 +910,21 @@
       <c r="Q2" s="1"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A3" s="28" t="s">
+      <c r="A3" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="29"/>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="30" t="s">
+      <c r="B3" s="24"/>
+      <c r="C3" s="24"/>
+      <c r="D3" s="24"/>
+      <c r="E3" s="25" t="s">
         <v>31</v>
       </c>
-      <c r="F3" s="30"/>
-      <c r="G3" s="30"/>
-      <c r="H3" s="30"/>
-      <c r="I3" s="30"/>
-      <c r="J3" s="30"/>
-      <c r="K3" s="30"/>
+      <c r="F3" s="25"/>
+      <c r="G3" s="25"/>
+      <c r="H3" s="25"/>
+      <c r="I3" s="25"/>
+      <c r="J3" s="25"/>
+      <c r="K3" s="25"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
       <c r="N3" s="1"/>
@@ -995,53 +1002,53 @@
       </c>
       <c r="Q5" s="1"/>
     </row>
-    <row r="6" spans="1:17" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A6" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="32" t="s">
         <v>33</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="D6" s="20" t="s">
+      <c r="D6" s="16" t="s">
         <v>35</v>
       </c>
-      <c r="E6" s="20" t="s">
+      <c r="E6" s="29" t="s">
         <v>36</v>
       </c>
-      <c r="F6" s="11" t="s">
+      <c r="F6" s="29" t="s">
         <v>37</v>
       </c>
-      <c r="G6" s="11" t="s">
+      <c r="G6" s="29" t="s">
         <v>38</v>
       </c>
-      <c r="H6" s="11" t="s">
+      <c r="H6" s="29" t="s">
         <v>39</v>
       </c>
-      <c r="I6" s="11" t="s">
+      <c r="I6" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="J6" s="11" t="s">
+      <c r="J6" s="29" t="s">
         <v>41</v>
       </c>
-      <c r="K6" s="11" t="s">
+      <c r="K6" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="L6" s="11" t="s">
+      <c r="L6" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="M6" s="12" t="s">
+      <c r="M6" s="30" t="s">
         <v>44</v>
       </c>
-      <c r="N6" s="11" t="s">
+      <c r="N6" s="29" t="s">
         <v>45</v>
       </c>
-      <c r="O6" s="11" t="s">
+      <c r="O6" s="29" t="s">
         <v>46</v>
       </c>
-      <c r="P6" s="13" t="s">
+      <c r="P6" s="31" t="s">
         <v>47</v>
       </c>
       <c r="Q6" s="1"/>
@@ -1051,57 +1058,57 @@
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
-      <c r="E7" s="14" t="s">
+      <c r="E7" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="F7" s="21" t="s">
+      <c r="F7" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="G7" s="21"/>
-      <c r="H7" s="21" t="s">
+      <c r="G7" s="17"/>
+      <c r="H7" s="17" t="s">
         <v>49</v>
       </c>
-      <c r="I7" s="21" t="s">
+      <c r="I7" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="J7" s="21" t="s">
+      <c r="J7" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="K7" s="21" t="s">
+      <c r="K7" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="L7" s="21" t="s">
+      <c r="L7" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="M7" s="21"/>
-      <c r="N7" s="21" t="s">
+      <c r="M7" s="17"/>
+      <c r="N7" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="O7" s="21" t="s">
+      <c r="O7" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="P7" s="22" t="s">
+      <c r="P7" s="18" t="s">
         <v>56</v>
       </c>
       <c r="Q7" s="1"/>
     </row>
     <row r="8" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="15"/>
-      <c r="B8" s="16"/>
-      <c r="C8" s="16"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="16"/>
-      <c r="F8" s="16"/>
-      <c r="G8" s="16"/>
-      <c r="H8" s="16"/>
-      <c r="I8" s="16"/>
-      <c r="J8" s="16"/>
-      <c r="K8" s="16"/>
-      <c r="L8" s="16"/>
-      <c r="M8" s="16"/>
-      <c r="N8" s="16"/>
-      <c r="O8" s="16"/>
-      <c r="P8" s="17"/>
+      <c r="A8" s="11"/>
+      <c r="B8" s="12"/>
+      <c r="C8" s="12"/>
+      <c r="D8" s="12"/>
+      <c r="E8" s="12"/>
+      <c r="F8" s="12"/>
+      <c r="G8" s="12"/>
+      <c r="H8" s="12"/>
+      <c r="I8" s="12"/>
+      <c r="J8" s="12"/>
+      <c r="K8" s="12"/>
+      <c r="L8" s="12"/>
+      <c r="M8" s="12"/>
+      <c r="N8" s="12"/>
+      <c r="O8" s="12"/>
+      <c r="P8" s="13"/>
       <c r="Q8" s="1"/>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.3">
@@ -1125,11 +1132,11 @@
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
-      <c r="B10" s="23" t="s">
+      <c r="B10" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="23"/>
-      <c r="D10" s="18" t="s">
+      <c r="C10" s="19"/>
+      <c r="D10" s="14" t="s">
         <v>57</v>
       </c>
       <c r="E10" s="1"/>
@@ -1148,11 +1155,11 @@
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
-      <c r="B11" s="23" t="s">
+      <c r="B11" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="23"/>
-      <c r="D11" s="18" t="s">
+      <c r="C11" s="19"/>
+      <c r="D11" s="14" t="s">
         <v>58</v>
       </c>
       <c r="E11" s="1"/>
@@ -1171,11 +1178,11 @@
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
-      <c r="B12" s="23" t="s">
+      <c r="B12" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="C12" s="23"/>
-      <c r="D12" s="18" t="s">
+      <c r="C12" s="19"/>
+      <c r="D12" s="14" t="s">
         <v>59</v>
       </c>
       <c r="E12" s="1"/>
@@ -1194,11 +1201,11 @@
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
-      <c r="B13" s="24" t="s">
+      <c r="B13" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="C13" s="24"/>
-      <c r="D13" s="19" t="s">
+      <c r="C13" s="26"/>
+      <c r="D13" s="15" t="s">
         <v>60</v>
       </c>
       <c r="E13" s="1"/>
@@ -1217,11 +1224,11 @@
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
-      <c r="B14" s="23" t="s">
+      <c r="B14" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="23"/>
-      <c r="D14" s="18" t="s">
+      <c r="C14" s="19"/>
+      <c r="D14" s="14" t="s">
         <v>61</v>
       </c>
       <c r="E14" s="1"/>
@@ -1240,11 +1247,11 @@
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
-      <c r="B15" s="23" t="s">
+      <c r="B15" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="C15" s="23"/>
-      <c r="D15" s="18" t="s">
+      <c r="C15" s="19"/>
+      <c r="D15" s="14" t="s">
         <v>62</v>
       </c>
       <c r="E15" s="1"/>
@@ -1263,11 +1270,11 @@
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
-      <c r="B16" s="23" t="s">
+      <c r="B16" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="C16" s="23"/>
-      <c r="D16" s="18" t="s">
+      <c r="C16" s="19"/>
+      <c r="D16" s="14" t="s">
         <v>63</v>
       </c>
       <c r="E16" s="1"/>
@@ -1286,11 +1293,11 @@
     </row>
     <row r="17" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
-      <c r="B17" s="23" t="s">
+      <c r="B17" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="C17" s="23"/>
-      <c r="D17" s="18" t="s">
+      <c r="C17" s="19"/>
+      <c r="D17" s="14" t="s">
         <v>64</v>
       </c>
       <c r="E17" s="1"/>
@@ -1309,11 +1316,11 @@
     </row>
     <row r="18" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
-      <c r="B18" s="23" t="s">
+      <c r="B18" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="C18" s="23"/>
-      <c r="D18" s="18" t="s">
+      <c r="C18" s="19"/>
+      <c r="D18" s="14" t="s">
         <v>65</v>
       </c>
       <c r="E18" s="1"/>
@@ -1332,11 +1339,11 @@
     </row>
     <row r="19" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
-      <c r="B19" s="24" t="s">
+      <c r="B19" s="26" t="s">
         <v>26</v>
       </c>
-      <c r="C19" s="24"/>
-      <c r="D19" s="19" t="s">
+      <c r="C19" s="26"/>
+      <c r="D19" s="15" t="s">
         <v>66</v>
       </c>
       <c r="E19" s="1"/>
@@ -1355,12 +1362,6 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="A1:P1"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="F2:J2"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="E3:K3"/>
     <mergeCell ref="B17:C17"/>
     <mergeCell ref="B18:C18"/>
     <mergeCell ref="B19:C19"/>
@@ -1370,6 +1371,12 @@
     <mergeCell ref="B14:C14"/>
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="F2:J2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="E3:K3"/>
   </mergeCells>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>

</xml_diff>